<commit_message>
auto: 更新 ETF Swing 2026-08-18
</commit_message>
<xml_diff>
--- a/hk_swing_pattern/ETF_Swing_Pattern.xlsx
+++ b/hk_swing_pattern/ETF_Swing_Pattern.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="swing" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="swing" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="指标说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'swing'!$A$1:$X$1</definedName>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.645</v>
+        <v>3.756</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>-9.34</v>
@@ -657,16 +657,16 @@
       <c r="S2" s="2" t="inlineStr"/>
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="n">
-        <v>22.74</v>
+        <v>23.93</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>7.68</v>
+        <v>9.1</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>1.75</v>
+        <v>4.25</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>0.06</v>
+        <v>2.58</v>
       </c>
     </row>
     <row r="3">
@@ -681,7 +681,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.479</v>
+        <v>1.501</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>101.66</v>
@@ -698,45 +698,49 @@
         <v>9</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="R3" s="2" t="inlineStr"/>
       <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="n">
-        <v>-8.130000000000001</v>
+        <v>-8.289999999999999</v>
       </c>
       <c r="V3" s="2" t="n">
-        <v>-6.13</v>
+        <v>-6.15</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-0.83</v>
+        <v>-1.61</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>0.23</v>
+        <v>-1.06</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.673</v>
+        <v>1.546</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>103.82</v>
+        <v>41.16</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
@@ -746,47 +750,49 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N4" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="inlineStr"/>
-      <c r="S4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="inlineStr"/>
+      <c r="T4" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U4" s="2" t="n">
-        <v>-28.24</v>
+        <v>25.27</v>
       </c>
       <c r="V4" s="2" t="n">
-        <v>-13.93</v>
+        <v>6.3</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>1.15</v>
+        <v>4.72</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>2.41</v>
+        <v>-2.82</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.52</v>
+        <v>0.927</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>41.16</v>
+        <v>96.56999999999999</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
@@ -806,43 +812,37 @@
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="inlineStr"/>
-      <c r="S5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="S5" s="2" t="inlineStr"/>
+      <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="n">
-        <v>23.76</v>
+        <v>1.95</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>6.16</v>
+        <v>4.01</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>4.46</v>
+        <v>0.34</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>0.32</v>
+        <v>4.47</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.918</v>
+        <v>3.052</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>96.56999999999999</v>
+        <v>76.81</v>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
@@ -852,51 +852,49 @@
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
-      <c r="Q6" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="R6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S6" s="2" t="inlineStr"/>
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="n">
-        <v>1.46</v>
+        <v>-0.63</v>
       </c>
       <c r="V6" s="2" t="n">
-        <v>4.56</v>
+        <v>-2.71</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.79</v>
+        <v>-1.42</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>6.88</v>
+        <v>-1.03</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3.021</v>
+        <v>4.801</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>76.81</v>
+        <v>6.93</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -908,47 +906,45 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="R7" s="2" t="n">
-        <v>-1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="R7" s="2" t="inlineStr"/>
       <c r="S7" s="2" t="inlineStr"/>
       <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="n">
-        <v>-0.36</v>
+        <v>5.14</v>
       </c>
       <c r="V7" s="2" t="n">
-        <v>-2.21</v>
+        <v>0</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>-0.77</v>
+        <v>0</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0.72</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.726</v>
+        <v>3.304</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>6.93</v>
+        <v>105.69</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
@@ -964,41 +960,45 @@
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
-      <c r="Q8" s="2" t="n">
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="R8" s="2" t="inlineStr"/>
       <c r="S8" s="2" t="inlineStr"/>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="n">
-        <v>4.86</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="V8" s="2" t="n">
-        <v>0</v>
+        <v>1.58</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>0</v>
+        <v>-1.17</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>0</v>
+        <v>-0.41</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7.998</v>
+        <v>0.522</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>-1.45</v>
+        <v>62.66</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
@@ -1010,47 +1010,47 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>预-1</t>
+          <t>预1</t>
         </is>
       </c>
       <c r="R9" s="2" t="inlineStr"/>
       <c r="S9" s="2" t="inlineStr"/>
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="n">
-        <v>15.43</v>
+        <v>-16.78</v>
       </c>
       <c r="V9" s="2" t="n">
-        <v>2.56</v>
+        <v>-9.23</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>0.48</v>
+        <v>-0.83</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>2.74</v>
+        <v>-3.12</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.296</v>
+        <v>0.401</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>105.69</v>
+        <v>110.32</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -1060,9 +1060,11 @@
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
@@ -1071,40 +1073,38 @@
           <t>预1</t>
         </is>
       </c>
-      <c r="R10" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R10" s="2" t="inlineStr"/>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="n">
-        <v>8.529999999999999</v>
+        <v>-6.03</v>
       </c>
       <c r="V10" s="2" t="n">
-        <v>2.9</v>
+        <v>0.37</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>1.18</v>
+        <v>-1.49</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>3.02</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.395</v>
+        <v>0.786</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>110.32</v>
+        <v>92.45</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1115,52 +1115,50 @@
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="n">
-        <v>-9</v>
+        <v>9</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
-      <c r="Q11" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="R11" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr"/>
       <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="n">
-        <v>-6.17</v>
+        <v>-14.1</v>
       </c>
       <c r="V11" s="2" t="n">
-        <v>0.32</v>
+        <v>-10.66</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>0.66</v>
+        <v>-1.66</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>6.52</v>
+        <v>-4.4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.782</v>
+        <v>3.225</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>92.45</v>
+        <v>-5.19</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1171,10 +1169,10 @@
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="n">
-        <v>9</v>
+        <v>-9</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
@@ -1183,34 +1181,34 @@
       <c r="S12" s="2" t="inlineStr"/>
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="n">
-        <v>-14.07</v>
+        <v>9.77</v>
       </c>
       <c r="V12" s="2" t="n">
-        <v>-9.800000000000001</v>
+        <v>-0.31</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>-0.76</v>
+        <v>2.11</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>-1.8</v>
+        <v>9.949999999999999</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>3.145</v>
+        <v>0.353</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>-5.19</v>
+        <v>108.28</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1224,49 +1222,47 @@
         <v>-9</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O13" s="2" t="n">
         <v>1</v>
       </c>
       <c r="P13" s="2" t="inlineStr"/>
-      <c r="Q13" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="Q13" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="R13" s="2" t="inlineStr"/>
       <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="n">
-        <v>8.44</v>
+        <v>-7.28</v>
       </c>
       <c r="V13" s="2" t="n">
-        <v>-1.25</v>
+        <v>-1.94</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>1.59</v>
+        <v>-0.43</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>4.98</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.351</v>
+        <v>1.172</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>108.28</v>
+        <v>6.23</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1276,51 +1272,47 @@
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O14" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="R14" s="2" t="inlineStr"/>
       <c r="S14" s="2" t="inlineStr"/>
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="n">
-        <v>-7.89</v>
+        <v>-3.51</v>
       </c>
       <c r="V14" s="2" t="n">
-        <v>-1.02</v>
+        <v>-12.15</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>2.38</v>
+        <v>-0.47</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>8.16</v>
+        <v>7.32</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.152</v>
+        <v>0.43</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>6.23</v>
+        <v>102.25</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1332,45 +1324,47 @@
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="R15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S15" s="2" t="inlineStr"/>
       <c r="T15" s="2" t="inlineStr"/>
       <c r="U15" s="2" t="n">
-        <v>-4.46</v>
+        <v>-39.55</v>
       </c>
       <c r="V15" s="2" t="n">
-        <v>-12.34</v>
+        <v>-20.2</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>0.6</v>
+        <v>-2.82</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>5.59</v>
+        <v>-0.15</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.441</v>
+        <v>1.238</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>102.25</v>
+        <v>17.98</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1382,7 +1376,7 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
@@ -1391,38 +1385,40 @@
       </c>
       <c r="R16" s="2" t="inlineStr"/>
       <c r="S16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" s="2" t="inlineStr"/>
+        <v>-1</v>
+      </c>
+      <c r="T16" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U16" s="2" t="n">
-        <v>-39.13</v>
+        <v>-1.76</v>
       </c>
       <c r="V16" s="2" t="n">
-        <v>-17.04</v>
+        <v>-3.63</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>2.23</v>
+        <v>-0.17</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>5.67</v>
+        <v>2.95</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.225</v>
+        <v>1.83</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>17.98</v>
+        <v>70.89</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1432,49 +1428,55 @@
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N17" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O17" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P17" s="2" t="inlineStr"/>
-      <c r="Q17" s="2" t="n">
-        <v>-1</v>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="R17" s="2" t="inlineStr"/>
-      <c r="S17" s="2" t="inlineStr"/>
-      <c r="T17" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="S17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" s="2" t="inlineStr"/>
       <c r="U17" s="2" t="n">
-        <v>-2.79</v>
+        <v>-28.69</v>
       </c>
       <c r="V17" s="2" t="n">
-        <v>-3.14</v>
+        <v>-12.12</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-0.24</v>
+        <v>-1.14</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>5.18</v>
+        <v>-0.41</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.094</v>
+        <v>2.274</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>100.94</v>
+        <v>-4.38</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -1486,45 +1488,47 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
-      <c r="Q18" s="2" t="inlineStr"/>
-      <c r="R18" s="2" t="n">
+      <c r="Q18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S18" s="2" t="inlineStr"/>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="n">
-        <v>-47.53</v>
+        <v>25.65</v>
       </c>
       <c r="V18" s="2" t="n">
-        <v>-21.58</v>
+        <v>14.29</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-3.66</v>
+        <v>-0.68</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>-0.25</v>
+        <v>4.48</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.822</v>
+        <v>1.699</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>70.89</v>
+        <v>-1.58</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1535,50 +1539,48 @@
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="n">
-        <v>-13</v>
+        <v>-9</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O19" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
-      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R19" s="2" t="inlineStr"/>
-      <c r="S19" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="n">
-        <v>-29.09</v>
+        <v>-6.04</v>
       </c>
       <c r="V19" s="2" t="n">
-        <v>-11.25</v>
+        <v>-8.359999999999999</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>0.88</v>
+        <v>0.09</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>0.53</v>
+        <v>6.73</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>2.264</v>
+        <v>1.117</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>-4.38</v>
+        <v>-12.75</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1588,51 +1590,47 @@
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N20" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
-      <c r="Q20" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="inlineStr"/>
       <c r="S20" s="2" t="inlineStr"/>
-      <c r="T20" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T20" s="2" t="inlineStr"/>
       <c r="U20" s="2" t="n">
-        <v>26.27</v>
+        <v>56.1</v>
       </c>
       <c r="V20" s="2" t="n">
-        <v>15.66</v>
+        <v>27.66</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>0.17</v>
+        <v>8.75</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>3.77</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.67</v>
+        <v>1.255</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>-1.58</v>
+        <v>20.27</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -1641,50 +1639,48 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L21" s="2" t="n">
+        <v>-13</v>
+      </c>
+      <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
-      <c r="Q21" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="Q21" s="2" t="inlineStr"/>
       <c r="R21" s="2" t="inlineStr"/>
       <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="n">
-        <v>-6.92</v>
+        <v>11.8</v>
       </c>
       <c r="V21" s="2" t="n">
-        <v>-8.460000000000001</v>
+        <v>5.59</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>0.85</v>
+        <v>-1.63</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>3.46</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.074</v>
+        <v>0.886</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>-12.75</v>
+        <v>-2.46</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
@@ -1693,48 +1689,50 @@
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L22" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
-      <c r="Q22" s="2" t="inlineStr"/>
+      <c r="Q22" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R22" s="2" t="inlineStr"/>
       <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="n">
-        <v>54.38</v>
+        <v>-6.72</v>
       </c>
       <c r="V22" s="2" t="n">
-        <v>25.02</v>
+        <v>-12.55</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>2.81</v>
+        <v>1.59</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-7.56</v>
+        <v>7.52</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.26</v>
+        <v>0.719</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>20.27</v>
+        <v>-13.75</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -1743,12 +1741,12 @@
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="n">
-        <v>-13</v>
-      </c>
-      <c r="M23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N23" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
@@ -1757,34 +1755,34 @@
       <c r="S23" s="2" t="inlineStr"/>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="n">
-        <v>12.74</v>
+        <v>53.6</v>
       </c>
       <c r="V23" s="2" t="n">
-        <v>7.72</v>
+        <v>24.46</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>2.71</v>
+        <v>10.65</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>7.31</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0.865</v>
+        <v>2.624</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>-2.46</v>
+        <v>-2.55</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -1796,47 +1794,49 @@
       <c r="L24" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="R24" s="2" t="inlineStr"/>
       <c r="S24" s="2" t="inlineStr"/>
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="n">
-        <v>-8.58</v>
+        <v>-4.98</v>
       </c>
       <c r="V24" s="2" t="n">
-        <v>-13.26</v>
+        <v>-10.06</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>0.33</v>
+        <v>0.75</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>4.52</v>
+        <v>7.84</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>1.023</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>-13.75</v>
+        <v>-11.11</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -1850,43 +1850,47 @@
         <v>-9</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
-      <c r="Q25" s="2" t="inlineStr"/>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="R25" s="2" t="inlineStr"/>
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="n">
-        <v>51.7</v>
+        <v>1.56</v>
       </c>
       <c r="V25" s="2" t="n">
-        <v>21.65</v>
+        <v>-3.81</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>4.54</v>
+        <v>0.34</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>-3.85</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>2.577</v>
+        <v>0.667</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>-2.55</v>
+        <v>103.82</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -1895,52 +1899,46 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="M26" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
-      <c r="Q26" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="Q26" s="2" t="inlineStr"/>
       <c r="R26" s="2" t="inlineStr"/>
       <c r="S26" s="2" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="n">
-        <v>-6.35</v>
+        <v>-28.41</v>
       </c>
       <c r="V26" s="2" t="n">
-        <v>-10.29</v>
+        <v>-15.91</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>0.91</v>
+        <v>-3.07</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>5.12</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1.001</v>
+        <v>8.196999999999999</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>-11.11</v>
+        <v>-1.45</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -1950,49 +1948,45 @@
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
-      <c r="Q27" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="Q27" s="2" t="inlineStr"/>
       <c r="R27" s="2" t="inlineStr"/>
       <c r="S27" s="2" t="inlineStr"/>
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="n">
-        <v>0.68</v>
+        <v>16.51</v>
       </c>
       <c r="V27" s="2" t="n">
-        <v>-4.4</v>
+        <v>3.44</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-1.35</v>
+        <v>0.93</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>0.8</v>
+        <v>5.99</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>588000 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>科创50ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1.814</v>
+        <v>1.205</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.14</v>
+        <v>-3.76</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2008,43 +2002,39 @@
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
-      <c r="Q28" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="inlineStr"/>
       <c r="S28" s="2" t="inlineStr"/>
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="n">
-        <v>28.31</v>
+        <v>46.38</v>
       </c>
       <c r="V28" s="2" t="n">
-        <v>14.01</v>
+        <v>26.06</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-1.79</v>
+        <v>2.98</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-6.36</v>
+        <v>-0.99</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.52</v>
+        <v>0.796</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>62.66</v>
+        <v>105.75</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2065,34 +2055,34 @@
       <c r="S29" s="2" t="inlineStr"/>
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="n">
-        <v>-17.24</v>
+        <v>-3.81</v>
       </c>
       <c r="V29" s="2" t="n">
-        <v>-8.25</v>
+        <v>-4.34</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>0.28</v>
+        <v>-1.24</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-1.7</v>
+        <v>-2.53</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.146</v>
+        <v>1.114</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>-3.76</v>
+        <v>100.94</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2104,7 +2094,7 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
@@ -2113,34 +2103,34 @@
       <c r="S30" s="2" t="inlineStr"/>
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="n">
-        <v>44.93</v>
+        <v>-48.44</v>
       </c>
       <c r="V30" s="2" t="n">
-        <v>22.05</v>
+        <v>-21.27</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-2.14</v>
+        <v>-4.39</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>-9.779999999999999</v>
+        <v>-1.84</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>588000 SH</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>科创50ETF</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.797</v>
+        <v>1.888</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>105.75</v>
+        <v>0.14</v>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr"/>
@@ -2152,7 +2142,7 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
@@ -2161,16 +2151,16 @@
       <c r="S31" s="2" t="inlineStr"/>
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="n">
-        <v>-2.96</v>
+        <v>29.53</v>
       </c>
       <c r="V31" s="2" t="n">
-        <v>-2.8</v>
+        <v>16.64</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>0.83</v>
+        <v>1.5</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>0.16</v>
+        <v>-2.5</v>
       </c>
     </row>
   </sheetData>
@@ -2201,7 +2191,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-08-14 | 30 只</t>
+          <t>截至: 2026-08-17 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 ETF Swing 2026-08-19
</commit_message>
<xml_diff>
--- a/hk_swing_pattern/ETF_Swing_Pattern.xlsx
+++ b/hk_swing_pattern/ETF_Swing_Pattern.xlsx
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.756</v>
+        <v>3.723</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>-9.34</v>
@@ -659,21 +659,25 @@
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S2" s="2" t="inlineStr"/>
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>23.93</v>
+        <v>24.91</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>9.1</v>
+        <v>8.32</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>4.25</v>
+        <v>2.72</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>2.58</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="3">
@@ -688,7 +692,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.501</v>
+        <v>1.5</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>101.66</v>
@@ -721,34 +725,34 @@
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-8.289999999999999</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-6.15</v>
+        <v>-5.88</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>-1.61</v>
+        <v>-1.42</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>-1.06</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>159981 SZ</t>
+          <t>159928 SZ</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>消费ETF</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1.546</v>
+        <v>0.671</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>41.16</v>
+        <v>103.82</v>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
@@ -758,50 +762,48 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="inlineStr"/>
       <c r="S4" s="2" t="inlineStr"/>
-      <c r="T4" s="2" t="inlineStr"/>
-      <c r="U4" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T4" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>25.27</v>
+        <v>-28.13</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>6.3</v>
+        <v>-15.04</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>4.72</v>
+        <v>-1.75</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>-2.82</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>159992 SZ</t>
+          <t>159981 SZ</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.927</v>
+        <v>1.563</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>96.56999999999999</v>
+        <v>41.16</v>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
@@ -823,36 +825,38 @@
       <c r="R5" s="2" t="inlineStr"/>
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
-      <c r="U5" s="2" t="inlineStr"/>
+      <c r="U5" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V5" s="2" t="n">
-        <v>1.95</v>
+        <v>26.24</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>4.01</v>
+        <v>7.78</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>0.34</v>
+        <v>2.44</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>4.47</v>
+        <v>4.22</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>510050 SH</t>
+          <t>159992 SZ</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>上证50ETF</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3.052</v>
+        <v>0.919</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>76.81</v>
+        <v>96.56999999999999</v>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
@@ -862,50 +866,56 @@
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="n">
+        <v>-13</v>
+      </c>
       <c r="N6" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S6" s="2" t="n">
-        <v>1</v>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>-0.63</v>
+        <v>2.42</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>-2.71</v>
+        <v>3.48</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>-1.42</v>
+        <v>-1.27</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>-1.03</v>
+        <v>5.75</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>510300 SH</t>
+          <t>510050 SH</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>沪深300ETF</t>
+          <t>上证50ETF</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4.801</v>
+        <v>3.047</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>6.93</v>
+        <v>76.81</v>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
@@ -917,46 +927,50 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
       <c r="R7" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S7" s="2" t="inlineStr"/>
-      <c r="T7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>5.14</v>
+        <v>-0.63</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>0</v>
+        <v>-2.58</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>0</v>
+        <v>-0.41</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>510300 SH</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>沪深300ETF</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>3.304</v>
+        <v>4.787</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>105.69</v>
+        <v>6.93</v>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
@@ -968,50 +982,46 @@
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S8" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" s="2" t="inlineStr"/>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>8.050000000000001</v>
+        <v>5.51</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>1.58</v>
+        <v>0</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>-1.17</v>
+        <v>0</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>-0.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.522</v>
+        <v>3.34</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>62.66</v>
+        <v>105.69</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
@@ -1023,48 +1033,48 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S9" s="2" t="inlineStr"/>
+      <c r="R9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>-16.78</v>
+        <v>7.99</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>-9.23</v>
+        <v>3</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>-0.83</v>
+        <v>-0.13</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>-3.12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.401</v>
+        <v>0.515</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>110.32</v>
+        <v>62.66</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -1075,7 +1085,7 @@
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="n">
-        <v>-9</v>
+        <v>13</v>
       </c>
       <c r="N10" s="2" t="n">
         <v>3</v>
@@ -1083,43 +1093,39 @@
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R10" s="2" t="inlineStr"/>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>-6.03</v>
+        <v>-16.84</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>0.37</v>
+        <v>-10.1</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>-1.49</v>
+        <v>-1.87</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>4.68</v>
+        <v>-1.89</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.786</v>
+        <v>0.401</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>92.45</v>
+        <v>110.32</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1130,10 +1136,10 @@
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="n">
-        <v>9</v>
+        <v>-9</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
@@ -1143,38 +1149,42 @@
           <t>预1</t>
         </is>
       </c>
-      <c r="S11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-14.1</v>
+        <v>-5.61</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-10.66</v>
+        <v>0.74</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>-1.66</v>
+        <v>-1.34</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>-4.4</v>
+        <v>7.72</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>3.225</v>
+        <v>0.777</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>-5.19</v>
+        <v>92.45</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1185,10 +1195,10 @@
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="n">
-        <v>-9</v>
+        <v>9</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
@@ -1198,34 +1208,34 @@
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>9.77</v>
+        <v>-14.31</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>-0.31</v>
+        <v>-11.35</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>2.11</v>
+        <v>-2.15</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>9.949999999999999</v>
+        <v>-2.48</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>0.353</v>
+        <v>3.213</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>108.28</v>
+        <v>-5.19</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1239,48 +1249,48 @@
         <v>-9</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O13" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="n">
-        <v>-1</v>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-7.28</v>
+        <v>10.82</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-1.94</v>
+        <v>-0.45</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>-0.43</v>
+        <v>1.67</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>6.1</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1.172</v>
+        <v>0.353</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>6.23</v>
+        <v>108.28</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1290,48 +1300,52 @@
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
       <c r="R14" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S14" s="2" t="inlineStr"/>
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>-3.51</v>
+        <v>-6.59</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-12.15</v>
+        <v>-1.57</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>-0.47</v>
+        <v>-0.25</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>7.32</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.43</v>
+        <v>1.169</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>102.25</v>
+        <v>6.23</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1343,48 +1357,46 @@
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
       <c r="R15" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S15" s="2" t="n">
-        <v>-1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="S15" s="2" t="inlineStr"/>
       <c r="T15" s="2" t="inlineStr"/>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-39.55</v>
+        <v>-2.3</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-20.2</v>
+        <v>-12.07</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>-2.82</v>
+        <v>0.8</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>-0.15</v>
+        <v>7.05</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.238</v>
+        <v>0.433</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>17.98</v>
+        <v>102.25</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1396,7 +1408,7 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
@@ -1404,42 +1416,40 @@
       <c r="R16" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S16" s="2" t="inlineStr"/>
-      <c r="T16" s="2" t="n">
+      <c r="S16" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="U16" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-1.76</v>
+        <v>-39.46</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-3.63</v>
+        <v>-19.28</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>-0.17</v>
+        <v>-1.8</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>2.95</v>
+        <v>4.21</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.83</v>
+        <v>1.229</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>70.89</v>
+        <v>17.98</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1449,56 +1459,48 @@
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O17" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="R17" s="2" t="inlineStr"/>
       <c r="S17" s="2" t="inlineStr"/>
       <c r="T17" s="2" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-28.69</v>
+        <v>-1.16</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-12.12</v>
+        <v>-4.05</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>-1.14</v>
+        <v>-0.51</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>-0.41</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>2.274</v>
+        <v>0.802</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>-4.38</v>
+        <v>105.75</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -1519,39 +1521,37 @@
         <v>1</v>
       </c>
       <c r="S18" s="2" t="inlineStr"/>
-      <c r="T18" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>25.65</v>
+        <v>-4.14</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>14.29</v>
+        <v>-3.25</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>-0.68</v>
+        <v>-0.51</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>4.48</v>
+        <v>3.37</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.699</v>
+        <v>1.116</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>-1.58</v>
+        <v>100.94</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1561,50 +1561,50 @@
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="n">
-        <v>1</v>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>-6.04</v>
+        <v>-49.96</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>-8.359999999999999</v>
+        <v>-20.77</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>0.09</v>
+        <v>-3.49</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>6.73</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.117</v>
+        <v>1.818</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>-12.75</v>
+        <v>70.89</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1615,47 +1615,49 @@
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="2" t="n">
-        <v>-9</v>
+        <v>-13</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="inlineStr"/>
       <c r="S20" s="2" t="inlineStr"/>
-      <c r="T20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>56.1</v>
+        <v>-28.42</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>27.66</v>
+        <v>-12.32</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>8.75</v>
+        <v>-1.1</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>1.63</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.255</v>
+        <v>2.239</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>20.27</v>
+        <v>-4.38</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -1664,49 +1666,55 @@
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="inlineStr"/>
-      <c r="S21" s="2" t="inlineStr"/>
-      <c r="T21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="T21" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>11.8</v>
+        <v>25.35</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>5.59</v>
+        <v>12.78</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>-1.63</v>
+        <v>-0.52</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>0</v>
+        <v>4.42</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0.886</v>
+        <v>1.684</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>-2.46</v>
+        <v>-1.58</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
@@ -1715,10 +1723,10 @@
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="M22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N22" s="2" t="n">
         <v>1</v>
       </c>
@@ -1726,40 +1734,40 @@
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-6.72</v>
+        <v>-5.49</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-12.55</v>
+        <v>-8.949999999999999</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>1.59</v>
+        <v>-0.36</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>7.52</v>
+        <v>5.23</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>0.719</v>
+        <v>1.101</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>-13.75</v>
+        <v>-12.75</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -1783,34 +1791,34 @@
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>53.6</v>
+        <v>57.92</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>24.46</v>
+        <v>25.86</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>10.65</v>
+        <v>6.69</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>3.56</v>
+        <v>-6.97</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>2.624</v>
+        <v>1.269</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>-2.55</v>
+        <v>20.27</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -1820,52 +1828,48 @@
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="M24" s="2" t="n">
-        <v>-9</v>
-      </c>
+        <v>-13</v>
+      </c>
+      <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="R24" s="2" t="inlineStr"/>
       <c r="S24" s="2" t="inlineStr"/>
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>-4.98</v>
+        <v>11.31</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-10.06</v>
+        <v>7.06</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>0.75</v>
+        <v>-0.73</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>7.84</v>
+        <v>6.34</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1.023</v>
+        <v>0.89</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>-11.11</v>
+        <v>-2.46</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -1874,53 +1878,51 @@
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr"/>
-      <c r="M25" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L25" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R25" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>1.56</v>
+        <v>-4.86</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>-3.81</v>
+        <v>-11.92</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>0.34</v>
+        <v>1.06</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>5.8</v>
+        <v>7.47</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>159928 SZ</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>消费ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.667</v>
+        <v>0.709</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>103.82</v>
+        <v>-13.75</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -1930,46 +1932,52 @@
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N26" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S26" s="2" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>-28.41</v>
+        <v>55.47</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>-15.91</v>
+        <v>22.76</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>-3.07</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-1.5</v>
+        <v>-4.49</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>8.196999999999999</v>
+        <v>2.616</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>-1.45</v>
+        <v>-2.55</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -1978,47 +1986,53 @@
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr"/>
-      <c r="M27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
       <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S27" s="2" t="inlineStr"/>
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>16.51</v>
+        <v>-3.89</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>3.44</v>
+        <v>-10.06</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>0.93</v>
+        <v>0.19</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>5.99</v>
+        <v>6.96</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1.205</v>
+        <v>1.037</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>-3.76</v>
+        <v>-11.11</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2028,46 +2042,52 @@
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N28" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr"/>
+      <c r="R28" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S28" s="2" t="inlineStr"/>
-      <c r="T28" s="2" t="inlineStr"/>
+      <c r="T28" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>46.38</v>
+        <v>2.06</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>26.06</v>
+        <v>-2.21</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>2.98</v>
+        <v>0.36</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-0.99</v>
+        <v>5.85</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>0.796</v>
+        <v>8.185</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>105.75</v>
+        <v>-1.45</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2079,7 +2099,7 @@
       <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -2089,34 +2109,34 @@
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-3.81</v>
+        <v>17.43</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-4.34</v>
+        <v>3.53</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-1.24</v>
+        <v>1.01</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>-2.53</v>
+        <v>4.27</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.114</v>
+        <v>1.202</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>100.94</v>
+        <v>-3.76</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2128,7 +2148,7 @@
       <c r="L30" s="2" t="inlineStr"/>
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
@@ -2138,16 +2158,16 @@
       <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-48.44</v>
+        <v>48.2</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-21.27</v>
+        <v>25.82</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>-4.39</v>
+        <v>3.77</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-1.84</v>
+        <v>-9.59</v>
       </c>
     </row>
     <row r="31">
@@ -2177,7 +2197,7 @@
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
@@ -2187,16 +2207,16 @@
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>29.53</v>
+        <v>31.03</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>16.64</v>
+        <v>16.8</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>1.5</v>
+        <v>2.89</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-2.5</v>
+        <v>-11.49</v>
       </c>
     </row>
   </sheetData>
@@ -2227,7 +2247,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-08-17 | 30 只</t>
+          <t>截至: 2026-08-18 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 ETF Swing 2026-08-20
</commit_message>
<xml_diff>
--- a/hk_swing_pattern/ETF_Swing_Pattern.xlsx
+++ b/hk_swing_pattern/ETF_Swing_Pattern.xlsx
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.723</v>
+        <v>3.498</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>-9.34</v>
@@ -659,25 +659,23 @@
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R2" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S2" s="2" t="inlineStr"/>
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>24.91</v>
+        <v>22.23</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>8.32</v>
+        <v>4.59</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>2.72</v>
+        <v>-2.12</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-1.9</v>
+        <v>-2.35</v>
       </c>
     </row>
     <row r="3">
@@ -692,7 +690,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.5</v>
+        <v>1.498</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>101.66</v>
@@ -716,25 +714,23 @@
       </c>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R3" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-8.630000000000001</v>
+        <v>-9.44</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-5.88</v>
+        <v>-3.24</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>-1.42</v>
+        <v>2.5</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>1.75</v>
+        <v>5.02</v>
       </c>
     </row>
     <row r="4">
@@ -749,7 +745,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.671</v>
+        <v>0.664</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>103.82</v>
@@ -764,7 +760,7 @@
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
@@ -776,16 +772,16 @@
       </c>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-28.13</v>
+        <v>-28.23</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-15.04</v>
+        <v>-13.4</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>-1.75</v>
+        <v>-0.11</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>2.56</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="5">
@@ -800,7 +796,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.563</v>
+        <v>1.567</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>41.16</v>
@@ -822,23 +818,27 @@
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>26.24</v>
+        <v>27.27</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>7.78</v>
+        <v>11.14</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>2.44</v>
+        <v>7.26</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>4.22</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="6">
@@ -853,7 +853,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.919</v>
+        <v>0.897</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>96.56999999999999</v>
@@ -870,15 +870,13 @@
         <v>-13</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R6" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
@@ -888,16 +886,16 @@
       <c r="T6" s="2" t="inlineStr"/>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>2.42</v>
+        <v>1.49</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>3.48</v>
+        <v>3.97</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>-1.27</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>5.75</v>
+        <v>5.64</v>
       </c>
     </row>
     <row r="7">
@@ -912,7 +910,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3.047</v>
+        <v>2.999</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>76.81</v>
@@ -936,23 +934,23 @@
         <v>-1</v>
       </c>
       <c r="S7" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="T7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>-0.63</v>
+        <v>-1.69</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>-2.58</v>
+        <v>-1.33</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>-0.8100000000000001</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>-0.41</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="8">
@@ -967,7 +965,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.787</v>
+        <v>4.654</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>6.93</v>
@@ -988,13 +986,13 @@
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
       <c r="R8" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S8" s="2" t="inlineStr"/>
       <c r="T8" s="2" t="inlineStr"/>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>5.51</v>
+        <v>4.21</v>
       </c>
       <c r="W8" s="2" t="n">
         <v>0</v>
@@ -1009,19 +1007,19 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>510880 SH</t>
+          <t>510500 SH</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>红利ETF</t>
+          <t>中证500ETF</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3.34</v>
+        <v>7.804</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>105.69</v>
+        <v>-1.45</v>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
@@ -1033,48 +1031,50 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S9" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
+      </c>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
       </c>
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>7.99</v>
+        <v>15.77</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>3</v>
+        <v>1.49</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>-0.13</v>
+        <v>-1.39</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>5</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>512000 SH</t>
+          <t>510880 SH</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>券商ETF</t>
+          <t>红利ETF</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.515</v>
+        <v>3.36</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>62.66</v>
+        <v>105.69</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
@@ -1084,48 +1084,50 @@
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="n">
-        <v>13</v>
-      </c>
+      <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
-      <c r="R10" s="2" t="inlineStr"/>
-      <c r="S10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>-16.84</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>-10.1</v>
+        <v>6.63</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>-1.87</v>
+        <v>4.07</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>-1.89</v>
+        <v>6.64</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>512010 SH</t>
+          <t>512000 SH</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>医药ETF</t>
+          <t>券商ETF</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.401</v>
+        <v>0.509</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>110.32</v>
+        <v>62.66</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
@@ -1136,7 +1138,7 @@
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="n">
-        <v>-9</v>
+        <v>13</v>
       </c>
       <c r="N11" s="2" t="n">
         <v>3</v>
@@ -1144,47 +1146,39 @@
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
       <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S11" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-5.61</v>
+        <v>-18.04</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>0.74</v>
+        <v>-8.5</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>-1.34</v>
+        <v>-0.34</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>7.72</v>
+        <v>-0.11</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>512070 SH</t>
+          <t>512010 SH</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>非银ETF</t>
+          <t>医药ETF</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.777</v>
+        <v>0.396</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>92.45</v>
+        <v>110.32</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -1195,47 +1189,51 @@
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="n">
-        <v>9</v>
+        <v>-9</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="inlineStr"/>
-      <c r="S12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-14.31</v>
+        <v>-6.09</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>-11.35</v>
+        <v>2.38</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>-2.15</v>
+        <v>1.15</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>-2.48</v>
+        <v>8.609999999999999</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>512100 SH</t>
+          <t>512070 SH</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>中证1000ETF</t>
+          <t>非银ETF</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>3.213</v>
+        <v>0.773</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>-5.19</v>
+        <v>92.45</v>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1246,51 +1244,47 @@
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="n">
-        <v>-9</v>
+        <v>9</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="R13" s="2" t="inlineStr"/>
       <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>10.82</v>
+        <v>-15.5</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-0.45</v>
+        <v>-9.19</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>1.67</v>
+        <v>-0.06</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>8.800000000000001</v>
+        <v>-1.16</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512170 SH</t>
+          <t>512100 SH</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>医疗ETF</t>
+          <t>中证1000ETF</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.353</v>
+        <v>3.048</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>108.28</v>
+        <v>-5.19</v>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
@@ -1304,48 +1298,50 @@
         <v>-9</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="O14" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
       <c r="R14" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>-6.59</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-1.57</v>
+        <v>-2.81</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>-0.25</v>
+        <v>-1.45</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>8.5</v>
+        <v>7.33</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>512660 SH</t>
+          <t>512170 SH</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>军工ETF</t>
+          <t>医疗ETF</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1.169</v>
+        <v>0.344</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>6.23</v>
+        <v>108.28</v>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
@@ -1355,48 +1351,54 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N15" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O15" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T15" s="2" t="inlineStr"/>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-2.3</v>
+        <v>-7.36</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-12.07</v>
+        <v>-1.24</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>0.8</v>
+        <v>0.67</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>7.05</v>
+        <v>8.609999999999999</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>512690 SH</t>
+          <t>512660 SH</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>酒ETF</t>
+          <t>军工ETF</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.433</v>
+        <v>1.108</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>102.25</v>
+        <v>6.23</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1408,7 +1410,7 @@
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
@@ -1416,40 +1418,44 @@
       <c r="R16" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S16" s="2" t="n">
+      <c r="S16" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
+      <c r="T16" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T16" s="2" t="inlineStr"/>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-39.46</v>
+        <v>-3.87</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-19.28</v>
+        <v>-14.2</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>-1.8</v>
+        <v>-1.63</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>4.21</v>
+        <v>5.01</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>512720 SH</t>
+          <t>512690 SH</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>计算机ETF</t>
+          <t>酒ETF</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1.229</v>
+        <v>0.425</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>17.98</v>
+        <v>102.25</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -1461,46 +1467,48 @@
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
       <c r="R17" s="2" t="inlineStr"/>
-      <c r="S17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T17" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-1.16</v>
+        <v>-39.93</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-4.05</v>
+        <v>-18.4</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>-0.51</v>
+        <v>-1.62</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>1.1</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>512800 SH</t>
+          <t>512720 SH</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>银行ETF</t>
+          <t>计算机ETF</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.802</v>
+        <v>1.162</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>105.75</v>
+        <v>17.98</v>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
@@ -1512,46 +1520,46 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
-      <c r="R18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr"/>
+      <c r="S18" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-4.14</v>
+        <v>-3.43</v>
       </c>
       <c r="W18" s="2" t="n">
+        <v>-6.66</v>
+      </c>
+      <c r="X18" s="2" t="n">
+        <v>-2.75</v>
+      </c>
+      <c r="Y18" s="2" t="n">
         <v>-3.25</v>
-      </c>
-      <c r="X18" s="2" t="n">
-        <v>-0.51</v>
-      </c>
-      <c r="Y18" s="2" t="n">
-        <v>3.37</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>513050 SH</t>
+          <t>512760 SH</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>中概互联ETF</t>
+          <t>半导体ETF</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.116</v>
+        <v>1.109</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>100.94</v>
+        <v>-3.76</v>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1563,48 +1571,46 @@
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
       <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="R19" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>-49.96</v>
+        <v>45.16</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>-20.77</v>
+        <v>19.21</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>-3.49</v>
+        <v>-4.11</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>1.2</v>
+        <v>-17.28</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>513090 SH</t>
+          <t>512800 SH</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>MSCI中国A50ETF</t>
+          <t>银行ETF</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1.818</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>70.89</v>
+        <v>105.75</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1614,50 +1620,54 @@
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
-      <c r="M20" s="2" t="n">
-        <v>-13</v>
-      </c>
+      <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="n">
         <v>2</v>
       </c>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
       <c r="Q20" s="2" t="inlineStr"/>
-      <c r="R20" s="2" t="inlineStr"/>
-      <c r="S20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-28.42</v>
+        <v>-3.91</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>-12.32</v>
+        <v>1.23</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>-1.1</v>
+        <v>4.29</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>0.39</v>
+        <v>6.22</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>513100 SH</t>
+          <t>513050 SH</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>纳指ETF</t>
+          <t>中概互联ETF</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2.239</v>
+        <v>1.114</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>-4.38</v>
+        <v>100.94</v>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
@@ -1667,54 +1677,48 @@
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr"/>
-      <c r="M21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="n">
+        <v>9</v>
+      </c>
       <c r="N21" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S21" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T21" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R21" s="2" t="inlineStr"/>
+      <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>25.35</v>
+        <v>-52.1</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>12.78</v>
+        <v>-18.53</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>-0.52</v>
+        <v>0.75</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>4.42</v>
+        <v>6.43</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>515030 SH</t>
+          <t>513090 SH</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>新能源车ETF</t>
+          <t>MSCI中国A50ETF</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.684</v>
+        <v>1.805</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>-1.58</v>
+        <v>70.89</v>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
@@ -1725,49 +1729,47 @@
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="n">
-        <v>-9</v>
+        <v>-13</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="R22" s="2" t="inlineStr"/>
       <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-5.49</v>
+        <v>-29.61</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-8.949999999999999</v>
+        <v>-10.32</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>-0.36</v>
+        <v>1.31</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>5.23</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>515050 SH</t>
+          <t>513100 SH</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>5GETF</t>
+          <t>纳指ETF</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1.101</v>
+        <v>2.2</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>-12.75</v>
+        <v>-4.38</v>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
@@ -1777,48 +1779,52 @@
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr"/>
-      <c r="M23" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
-      <c r="R23" s="2" t="inlineStr"/>
-      <c r="S23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>57.92</v>
+        <v>23.73</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>25.86</v>
+        <v>13.93</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>6.69</v>
+        <v>0.61</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>-6.97</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>515220 SH</t>
+          <t>515030 SH</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>煤炭ETF</t>
+          <t>新能源车ETF</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.269</v>
+        <v>1.631</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>20.27</v>
+        <v>-1.58</v>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
@@ -1827,49 +1833,55 @@
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="n">
-        <v>-13</v>
-      </c>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr"/>
-      <c r="S24" s="2" t="inlineStr"/>
+      <c r="R24" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T24" s="2" t="inlineStr"/>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>11.31</v>
+        <v>-7.21</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>7.06</v>
+        <v>-9.31</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-0.73</v>
+        <v>-0.98</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>6.34</v>
+        <v>5.94</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>515790 SH</t>
+          <t>515050 SH</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>光伏ETF</t>
+          <t>5GETF</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.89</v>
+        <v>1.012</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>-2.46</v>
+        <v>-12.75</v>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
@@ -1878,51 +1890,51 @@
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="M25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N25" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
       <c r="R25" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>-4.86</v>
+        <v>54.43</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>-11.92</v>
+        <v>18.73</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>1.06</v>
+        <v>-3.27</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>7.47</v>
+        <v>-8.710000000000001</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>515880 SH</t>
+          <t>515220 SH</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>通信ETF</t>
+          <t>煤炭ETF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.709</v>
+        <v>1.273</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>-13.75</v>
+        <v>20.27</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -1931,12 +1943,12 @@
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="L26" s="2" t="n">
+        <v>-13</v>
+      </c>
+      <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
@@ -1950,34 +1962,34 @@
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>55.47</v>
+        <v>11.45</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>22.76</v>
+        <v>10.42</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>8.119999999999999</v>
+        <v>4.19</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>-4.49</v>
+        <v>6.47</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>516160 SH</t>
+          <t>515790 SH</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>新能源ETF</t>
+          <t>光伏ETF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>2.616</v>
+        <v>0.845</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>-2.55</v>
+        <v>-2.46</v>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr"/>
@@ -1989,9 +2001,7 @@
       <c r="L27" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="M27" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
         <v>1</v>
       </c>
@@ -2001,38 +2011,42 @@
       <c r="R27" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T27" s="2" t="inlineStr"/>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-3.89</v>
+        <v>-6.34</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-10.06</v>
+        <v>-13.98</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>0.19</v>
+        <v>-2.03</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>6.96</v>
+        <v>4.52</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>562500 SH</t>
+          <t>515880 SH</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>碳中和ETF</t>
+          <t>通信ETF</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1.037</v>
+        <v>0.652</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>-11.11</v>
+        <v>-13.75</v>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
@@ -2046,48 +2060,46 @@
         <v>-9</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S28" s="2" t="inlineStr"/>
-      <c r="T28" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>2.06</v>
+        <v>52.41</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>-2.21</v>
+        <v>15.86</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>0.36</v>
+        <v>-1.39</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>5.85</v>
+        <v>-6.17</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>510500 SH</t>
+          <t>516160 SH</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>中证500ETF</t>
+          <t>新能源ETF</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>8.185</v>
+        <v>2.514</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>-1.45</v>
+        <v>-2.55</v>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr"/>
@@ -2096,47 +2108,57 @@
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="inlineStr"/>
       <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr"/>
-      <c r="M29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N29" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="inlineStr"/>
-      <c r="S29" s="2" t="inlineStr"/>
+      <c r="R29" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S29" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="T29" s="2" t="inlineStr"/>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>17.43</v>
+        <v>-5.55</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>3.53</v>
+        <v>-11.17</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>1.01</v>
+        <v>-1.31</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>4.27</v>
+        <v>6.03</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>512760 SH</t>
+          <t>562500 SH</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>半导体ETF</t>
+          <t>碳中和ETF</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1.202</v>
+        <v>0.956</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>-3.76</v>
+        <v>-11.11</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -2146,28 +2168,34 @@
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N30" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
       <c r="Q30" s="2" t="inlineStr"/>
-      <c r="R30" s="2" t="inlineStr"/>
+      <c r="R30" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S30" s="2" t="inlineStr"/>
-      <c r="T30" s="2" t="inlineStr"/>
+      <c r="T30" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>48.2</v>
+        <v>-0.63</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>25.82</v>
+        <v>-7.23</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>3.77</v>
+        <v>-3.79</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>-9.59</v>
+        <v>1.99</v>
       </c>
     </row>
     <row r="31">
@@ -2182,7 +2210,7 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.888</v>
+        <v>1.761</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>0.14</v>
@@ -2202,21 +2230,23 @@
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="inlineStr"/>
-      <c r="R31" s="2" t="inlineStr"/>
+      <c r="R31" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="S31" s="2" t="inlineStr"/>
       <c r="T31" s="2" t="inlineStr"/>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>31.03</v>
+        <v>28.21</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>16.8</v>
+        <v>11.93</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>2.89</v>
+        <v>-3.05</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-11.49</v>
+        <v>-12.84</v>
       </c>
     </row>
   </sheetData>
@@ -2247,7 +2277,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-08-18 | 30 只</t>
+          <t>截至: 2026-08-19 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 ETF Swing 2026-08-21
</commit_message>
<xml_diff>
--- a/hk_swing_pattern/ETF_Swing_Pattern.xlsx
+++ b/hk_swing_pattern/ETF_Swing_Pattern.xlsx
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3.498</v>
+        <v>3.512</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>-9.34</v>
@@ -666,16 +666,16 @@
       <c r="T2" s="2" t="inlineStr"/>
       <c r="U2" s="2" t="inlineStr"/>
       <c r="V2" s="2" t="n">
-        <v>22.23</v>
+        <v>19.74</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>4.59</v>
+        <v>4.92</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>-2.12</v>
+        <v>-1.6</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>-2.35</v>
+        <v>-1.73</v>
       </c>
     </row>
     <row r="3">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1.498</v>
+        <v>1.516</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>101.66</v>
@@ -707,30 +707,32 @@
         <v>9</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
-        <v>-9.44</v>
+        <v>-9.6</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>-3.24</v>
+        <v>-2</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>2.5</v>
+        <v>3.41</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>5.02</v>
+        <v>5.38</v>
       </c>
     </row>
     <row r="4">
@@ -745,7 +747,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.664</v>
+        <v>0.669</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>103.82</v>
@@ -765,23 +767,25 @@
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S4" s="2" t="inlineStr"/>
-      <c r="T4" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T4" s="2" t="inlineStr"/>
       <c r="U4" s="2" t="inlineStr"/>
       <c r="V4" s="2" t="n">
-        <v>-28.23</v>
+        <v>-28.5</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>-13.4</v>
+        <v>-12.62</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>-0.11</v>
+        <v>0.08</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>3.2</v>
+        <v>4.62</v>
       </c>
     </row>
     <row r="5">
@@ -796,7 +800,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.567</v>
+        <v>1.564</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>41.16</v>
@@ -813,7 +817,7 @@
         <v>-13</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
@@ -825,20 +829,18 @@
       </c>
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
-      <c r="U5" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="U5" s="2" t="inlineStr"/>
       <c r="V5" s="2" t="n">
-        <v>27.27</v>
+        <v>27.82</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>11.14</v>
+        <v>10.94</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>7.26</v>
+        <v>6.13</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>5.5</v>
+        <v>4.94</v>
       </c>
     </row>
     <row r="6">
@@ -853,7 +855,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.897</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>96.56999999999999</v>
@@ -861,41 +863,51 @@
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="n">
         <v>-13</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="S6" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U6" s="2" t="inlineStr"/>
       <c r="V6" s="2" t="n">
-        <v>1.49</v>
+        <v>1.21</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>3.97</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>-0.07000000000000001</v>
+        <v>2.79</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>5.64</v>
+        <v>10.86</v>
       </c>
     </row>
     <row r="7">
@@ -910,7 +922,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.999</v>
+        <v>2.988</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>76.81</v>
@@ -936,21 +948,19 @@
       <c r="S7" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T7" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr"/>
       <c r="V7" s="2" t="n">
-        <v>-1.69</v>
+        <v>-2.98</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>-1.33</v>
+        <v>-1.64</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.16</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>0.13</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="8">
@@ -965,7 +975,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.654</v>
+        <v>4.653</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>6.93</v>
@@ -989,10 +999,12 @@
         <v>-1</v>
       </c>
       <c r="S8" s="2" t="inlineStr"/>
-      <c r="T8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U8" s="2" t="inlineStr"/>
       <c r="V8" s="2" t="n">
-        <v>4.21</v>
+        <v>2.79</v>
       </c>
       <c r="W8" s="2" t="n">
         <v>0</v>
@@ -1016,7 +1028,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7.804</v>
+        <v>7.863</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>-1.45</v>
@@ -1031,7 +1043,7 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
@@ -1039,24 +1051,20 @@
       <c r="R9" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S9" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="S9" s="2" t="inlineStr"/>
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr"/>
       <c r="V9" s="2" t="n">
-        <v>15.77</v>
+        <v>14.35</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>1.49</v>
+        <v>2.23</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>-1.39</v>
+        <v>-0.08</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>2.48</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="10">
@@ -1071,7 +1079,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3.36</v>
+        <v>3.382</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>105.69</v>
@@ -1100,16 +1108,16 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr"/>
       <c r="V10" s="2" t="n">
-        <v>8.220000000000001</v>
+        <v>8.99</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>6.63</v>
+        <v>7.37</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>4.07</v>
+        <v>5.29</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>6.64</v>
+        <v>6.96</v>
       </c>
     </row>
     <row r="11">
@@ -1124,7 +1132,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>0.509</v>
+        <v>0.508</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>62.66</v>
@@ -1151,16 +1159,16 @@
       <c r="T11" s="2" t="inlineStr"/>
       <c r="U11" s="2" t="inlineStr"/>
       <c r="V11" s="2" t="n">
-        <v>-18.04</v>
+        <v>-19.77</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>-8.5</v>
+        <v>-8.57</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>-0.34</v>
+        <v>-1.22</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>-0.11</v>
+        <v>-1.03</v>
       </c>
     </row>
     <row r="12">
@@ -1175,7 +1183,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.396</v>
+        <v>0.4</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>110.32</v>
@@ -1198,24 +1206,24 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="inlineStr"/>
-      <c r="S12" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U12" s="2" t="inlineStr"/>
       <c r="V12" s="2" t="n">
-        <v>-6.09</v>
+        <v>-6.78</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>2.38</v>
+        <v>3.53</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>1.15</v>
+        <v>1.81</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>8.609999999999999</v>
+        <v>10.12</v>
       </c>
     </row>
     <row r="13">
@@ -1252,21 +1260,25 @@
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
       <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="n">
-        <v>-15.5</v>
+        <v>-16.81</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>-9.19</v>
+        <v>-9.08</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>-0.06</v>
+        <v>-0.52</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>-1.16</v>
+        <v>-1.61</v>
       </c>
     </row>
     <row r="14">
@@ -1281,7 +1293,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>3.048</v>
+        <v>3.074</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>-5.19</v>
@@ -1298,7 +1310,7 @@
         <v>-9</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
@@ -1306,24 +1318,20 @@
       <c r="R14" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S14" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="S14" s="2" t="inlineStr"/>
       <c r="T14" s="2" t="inlineStr"/>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="n">
-        <v>9.130000000000001</v>
+        <v>7.86</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>-2.81</v>
+        <v>-2.02</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>-1.45</v>
+        <v>-0.12</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>7.33</v>
+        <v>7.77</v>
       </c>
     </row>
     <row r="15">
@@ -1338,7 +1346,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0.344</v>
+        <v>0.359</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>108.28</v>
@@ -1347,9 +1355,15 @@
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr"/>
       <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="n">
         <v>-9</v>
@@ -1362,25 +1376,25 @@
       </c>
       <c r="P15" s="2" t="inlineStr"/>
       <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr"/>
-      <c r="S15" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr"/>
       <c r="T15" s="2" t="inlineStr"/>
       <c r="U15" s="2" t="inlineStr"/>
       <c r="V15" s="2" t="n">
-        <v>-7.36</v>
+        <v>-7.5</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>-1.24</v>
+        <v>3.17</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>0.67</v>
+        <v>3.26</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>8.609999999999999</v>
+        <v>13.89</v>
       </c>
     </row>
     <row r="16">
@@ -1395,7 +1409,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1.108</v>
+        <v>1.097</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>6.23</v>
@@ -1418,26 +1432,22 @@
       <c r="R16" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S16" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="S16" s="2" t="inlineStr"/>
       <c r="T16" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>-3.87</v>
+        <v>-5.71</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-14.2</v>
+        <v>-14.95</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>-1.63</v>
+        <v>-2.19</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>5.01</v>
+        <v>3.23</v>
       </c>
     </row>
     <row r="17">
@@ -1452,7 +1462,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.425</v>
+        <v>0.426</v>
       </c>
       <c r="D17" s="2" t="n">
         <v>102.25</v>
@@ -1473,24 +1483,22 @@
       <c r="P17" s="2" t="inlineStr"/>
       <c r="Q17" s="2" t="inlineStr"/>
       <c r="R17" s="2" t="inlineStr"/>
-      <c r="S17" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="S17" s="2" t="inlineStr"/>
       <c r="T17" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="U17" s="2" t="inlineStr"/>
       <c r="V17" s="2" t="n">
-        <v>-39.93</v>
+        <v>-40.71</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>-18.4</v>
+        <v>-18.03</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>-1.62</v>
+        <v>-2.28</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>3.64</v>
+        <v>5.18</v>
       </c>
     </row>
     <row r="18">
@@ -1505,7 +1513,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1.162</v>
+        <v>1.163</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>17.98</v>
@@ -1520,7 +1528,7 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
@@ -1532,16 +1540,16 @@
       <c r="T18" s="2" t="inlineStr"/>
       <c r="U18" s="2" t="inlineStr"/>
       <c r="V18" s="2" t="n">
-        <v>-3.43</v>
+        <v>-6.07</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>-6.66</v>
+        <v>-6.54</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>-2.75</v>
+        <v>-3.03</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>-3.25</v>
+        <v>-0.72</v>
       </c>
     </row>
     <row r="19">
@@ -1556,7 +1564,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1.109</v>
+        <v>1.099</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>-3.76</v>
@@ -1583,16 +1591,16 @@
       <c r="T19" s="2" t="inlineStr"/>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="n">
-        <v>45.16</v>
+        <v>41.94</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>19.21</v>
+        <v>17.95</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>-4.11</v>
+        <v>-3.62</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>-17.28</v>
+        <v>-12.07</v>
       </c>
     </row>
     <row r="20">
@@ -1607,7 +1615,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.8149999999999999</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>105.75</v>
@@ -1630,26 +1638,22 @@
       <c r="R20" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="S20" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="S20" s="2" t="inlineStr"/>
       <c r="T20" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="n">
-        <v>-3.91</v>
+        <v>-3.78</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>1.23</v>
+        <v>1.7</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>4.29</v>
+        <v>3.93</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>6.22</v>
+        <v>6.53</v>
       </c>
     </row>
     <row r="21">
@@ -1664,7 +1668,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.114</v>
+        <v>1.131</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>100.94</v>
@@ -1686,21 +1690,25 @@
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="2" t="inlineStr"/>
       <c r="U21" s="2" t="inlineStr"/>
       <c r="V21" s="2" t="n">
-        <v>-52.1</v>
+        <v>-53.33</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>-18.53</v>
+        <v>-17.14</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>0.75</v>
+        <v>3.12</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>6.43</v>
+        <v>7.15</v>
       </c>
     </row>
     <row r="22">
@@ -1715,7 +1723,7 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.805</v>
+        <v>1.814</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>70.89</v>
@@ -1737,21 +1745,25 @@
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
       <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr"/>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="n">
-        <v>-29.61</v>
+        <v>-31.37</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>-10.32</v>
+        <v>-9.73</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>1.31</v>
+        <v>1.08</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>1.9</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="23">
@@ -1766,7 +1778,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>2.2</v>
+        <v>2.212</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>-4.38</v>
@@ -1789,24 +1801,20 @@
       <c r="R23" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S23" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="S23" s="2" t="inlineStr"/>
       <c r="T23" s="2" t="inlineStr"/>
       <c r="U23" s="2" t="inlineStr"/>
       <c r="V23" s="2" t="n">
-        <v>23.73</v>
+        <v>22.25</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>13.93</v>
+        <v>14.49</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>0.61</v>
+        <v>0.79</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>5.1</v>
+        <v>6.15</v>
       </c>
     </row>
     <row r="24">
@@ -1821,7 +1829,7 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1.631</v>
+        <v>1.619</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>-1.58</v>
@@ -1846,24 +1854,22 @@
       <c r="R24" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S24" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U24" s="2" t="inlineStr"/>
       <c r="V24" s="2" t="n">
-        <v>-7.21</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>-9.31</v>
+        <v>-9.99</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>-0.98</v>
+        <v>-0.95</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>5.94</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="25">
@@ -1878,7 +1884,7 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1.012</v>
+        <v>1.023</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>-12.75</v>
@@ -1895,7 +1901,7 @@
         <v>-9</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
@@ -1907,16 +1913,16 @@
       <c r="T25" s="2" t="inlineStr"/>
       <c r="U25" s="2" t="inlineStr"/>
       <c r="V25" s="2" t="n">
-        <v>54.43</v>
+        <v>50.95</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>18.73</v>
+        <v>19.77</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>-3.27</v>
+        <v>-2.09</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>-8.710000000000001</v>
+        <v>-6.27</v>
       </c>
     </row>
     <row r="26">
@@ -1931,7 +1937,7 @@
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1.273</v>
+        <v>1.268</v>
       </c>
       <c r="D26" s="2" t="n">
         <v>20.27</v>
@@ -1948,30 +1954,28 @@
       </c>
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
       <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="R26" s="2" t="n">
+        <v>-1</v>
       </c>
       <c r="S26" s="2" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr"/>
       <c r="U26" s="2" t="inlineStr"/>
       <c r="V26" s="2" t="n">
-        <v>11.45</v>
+        <v>12.53</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>10.42</v>
+        <v>10.01</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>4.19</v>
+        <v>4.06</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>6.47</v>
+        <v>5.36</v>
       </c>
     </row>
     <row r="27">
@@ -1986,7 +1990,7 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0.845</v>
+        <v>0.849</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>-2.46</v>
@@ -2003,7 +2007,7 @@
       </c>
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
@@ -2011,24 +2015,22 @@
       <c r="R27" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S27" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="inlineStr"/>
+      <c r="T27" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U27" s="2" t="inlineStr"/>
       <c r="V27" s="2" t="n">
-        <v>-6.34</v>
+        <v>-7.42</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>-13.98</v>
+        <v>-13.56</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>-2.03</v>
+        <v>-0.05</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>4.52</v>
+        <v>3.43</v>
       </c>
     </row>
     <row r="28">
@@ -2043,7 +2045,7 @@
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0.652</v>
+        <v>0.664</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>-13.75</v>
@@ -2060,7 +2062,7 @@
         <v>-9</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
@@ -2072,16 +2074,16 @@
       <c r="T28" s="2" t="inlineStr"/>
       <c r="U28" s="2" t="inlineStr"/>
       <c r="V28" s="2" t="n">
-        <v>52.41</v>
+        <v>49.47</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>15.86</v>
+        <v>17.74</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>-1.39</v>
+        <v>0.12</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>-6.17</v>
+        <v>-3.4</v>
       </c>
     </row>
     <row r="29">
@@ -2096,7 +2098,7 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>2.514</v>
+        <v>2.497</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>-2.55</v>
@@ -2123,24 +2125,22 @@
       <c r="R29" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="S29" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
-      <c r="T29" s="2" t="inlineStr"/>
+      <c r="S29" s="2" t="inlineStr"/>
+      <c r="T29" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="n">
-        <v>-5.55</v>
+        <v>-7.24</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>-11.17</v>
+        <v>-11.75</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>-1.31</v>
+        <v>-1.09</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>6.03</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="30">
@@ -2155,7 +2155,7 @@
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.956</v>
+        <v>0.952</v>
       </c>
       <c r="D30" s="2" t="n">
         <v>-11.11</v>
@@ -2172,7 +2172,7 @@
         <v>-9</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
@@ -2181,21 +2181,19 @@
         <v>-1</v>
       </c>
       <c r="S30" s="2" t="inlineStr"/>
-      <c r="T30" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="T30" s="2" t="inlineStr"/>
       <c r="U30" s="2" t="inlineStr"/>
       <c r="V30" s="2" t="n">
-        <v>-0.63</v>
+        <v>-2.96</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>-7.23</v>
+        <v>-7.56</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>-3.79</v>
+        <v>-2.89</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>1.99</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="31">
@@ -2210,7 +2208,7 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1.761</v>
+        <v>1.744</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>0.14</v>
@@ -2234,19 +2232,21 @@
         <v>-1</v>
       </c>
       <c r="S31" s="2" t="inlineStr"/>
-      <c r="T31" s="2" t="inlineStr"/>
+      <c r="T31" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U31" s="2" t="inlineStr"/>
       <c r="V31" s="2" t="n">
-        <v>28.21</v>
+        <v>25.16</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>11.93</v>
+        <v>10.73</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>-3.05</v>
+        <v>-3.23</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>-12.84</v>
+        <v>-9.01</v>
       </c>
     </row>
   </sheetData>
@@ -2277,7 +2277,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-08-19 | 30 只</t>
+          <t>截至: 2026-08-20 | 30 只</t>
         </is>
       </c>
     </row>

</xml_diff>